<commit_message>
Update excel master data
</commit_message>
<xml_diff>
--- a/excel_data/bank_name.xlsx
+++ b/excel_data/bank_name.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://pixeltruth-my.sharepoint.com/personal/shubhankar_shukla_pixeltruth_com/Documents/Python_Codes/IS_Dashboard/excel_data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://pixeltruth-my.sharepoint.com/personal/shubhankar_shukla_pixeltruth_com/Documents/Python_Codes/Testing_Code/excel_data/"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="8" documentId="8_{B90F617B-F823-4302-8087-77E1928040CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8298661B-4F84-4914-BE68-B69326E94704}"/>

</xml_diff>

<commit_message>
Updated app, bank data and UI
</commit_message>
<xml_diff>
--- a/excel_data/bank_name.xlsx
+++ b/excel_data/bank_name.xlsx
@@ -1,20 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://pixeltruth-my.sharepoint.com/personal/shubhankar_shukla_pixeltruth_com/Documents/Code_Hub/Testing_Code/excel_data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="14" documentId="8_{B90F617B-F823-4302-8087-77E1928040CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{51E77912-0DD8-46AE-BE4C-A9E62EE71C80}"/>
+  <xr:revisionPtr revIDLastSave="19" documentId="8_{B90F617B-F823-4302-8087-77E1928040CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D8557D2D-943F-4F25-9600-D20A95C5E791}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{52E78C5D-4E12-44D1-A43B-C09912A5A9A0}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$B$496</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -6685,6 +6688,7 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:B496" xr:uid="{71C0A434-7324-4CF0-BE95-1E232476045C}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>